<commit_message>
Set recommended tariff prices: 690 / 1 690 / from 4 900 RUB per month
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ADSquzsspwAL5eKo1c74of
</commit_message>
<xml_diff>
--- a/lawtracker-economics.xlsx
+++ b/lawtracker-economics.xlsx
@@ -834,11 +834,11 @@
         </is>
       </c>
       <c r="B6" s="12" t="n">
-        <v>990</v>
+        <v>690</v>
       </c>
       <c r="C6" s="9" t="inlineStr">
         <is>
-          <t>Предварительная цена с сайта (раздел «Тарифы»), не утверждена</t>
+          <t>Рекомендованная цена с сайта (раздел «Тарифы»); ориентир — конкурент от ~3 500 ₽/мес; не утверждена</t>
         </is>
       </c>
     </row>
@@ -849,11 +849,11 @@
         </is>
       </c>
       <c r="B7" s="12" t="n">
-        <v>2990</v>
+        <v>1690</v>
       </c>
       <c r="C7" s="9" t="inlineStr">
         <is>
-          <t>Предварительная цена с сайта, не утверждена</t>
+          <t>Рекомендованная цена с сайта; не утверждена</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Economics: minimal scenario is a lean beta (hosting and mailings only, AI on free GigaChat tokens)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ADSquzsspwAL5eKo1c74of
</commit_message>
<xml_diff>
--- a/lawtracker-economics.xlsx
+++ b/lawtracker-economics.xlsx
@@ -1,18 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Итоги" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Допущения" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Расходы" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Прогноз_мин" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Прогноз_реал" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Безубыточность" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Итоги" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Допущения" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Расходы" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прогноз_мин" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Прогноз_реал" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Безубыточность" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -217,6 +217,46 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/comments/comment1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <authors>
+    <author>Claude</author>
+  </authors>
+  <commentList>
+    <comment ref="B14" authorId="0" shapeId="0">
+      <text>
+        <t>Бета-версия: самый дешёвый VPS в РФ. По рейтингам 2026 года тарифы стартуют примерно от 180–260 ₽/мес (Cloud4box, Aeza, Beget ≈210 ₽). Закладываю 300 ₽. Если для PostgreSQL, pgvector и Airflow не хватит памяти, понадобится сервер за 500–1 000 ₽. Цены из агрегаторов, проверить у провайдера.</t>
+      </text>
+    </comment>
+    <comment ref="B15" authorId="0" shapeId="0">
+      <text>
+        <t>ИИ-разбор на бета-версии идёт на бесплатных токенах GigaChat (Freemium: по документации Сбера 365 млн токенов, физлицо, один поток). Условия для новых клиентов после 01.09.2026 проверить при регистрации. Когда токены закончатся, расход берёт на себя «переменная» строка (60 ₽ на пользователя) на листе «Допущения».</t>
+      </text>
+    </comment>
+    <comment ref="B16" authorId="0" shapeId="0">
+      <text>
+        <t>Рассылки: платный тариф «Лайт» UniSender ≈770 ₽/мес (цена из стороннего каталога, не с официального сайта). Бесплатный тариф («Фри»: 1 500 писем на 100 контактов) покрывает бета-тест 30–50 компаний, тогда строка может быть 0.</t>
+      </text>
+    </comment>
+    <comment ref="B17" authorId="0" shapeId="0">
+      <text>
+        <t>Бета-версия: юрист-эксперт без оплаты (помогает университет или команда).</t>
+      </text>
+    </comment>
+    <comment ref="B21" authorId="0" shapeId="0">
+      <text>
+        <t>Бета-версия: бухгалтерия силами команды, расход не закладывается.</t>
+      </text>
+    </comment>
+    <comment ref="B22" authorId="0" shapeId="0">
+      <text>
+        <t>Бета-версия: без рекламы, пилотные компании привлекаются через университет и партнёров.</t>
+      </text>
+    </comment>
+  </commentList>
+</comments>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1106,7 +1146,7 @@
     <row r="2" ht="40" customHeight="1">
       <c r="A2" s="9" t="inlineStr">
         <is>
-          <t>Две колонки сценариев: «Минимальный» (основатели без зарплат, юрист почасово) и «Реалистичный» (небольшая команда без разработчиков). «Облагается взносами» = 1, если это зарплата штатного сотрудника.</t>
+          <t>Две колонки сценариев: «Минимальный» — бета-версия: ежемесячно только хостинг и рассылки, ИИ на бесплатных токенах GigaChat, основатели без зарплат, юрист и бухгалтер без оплаты; «Реалистичный» — небольшая команда без разработчиков (не менялся). «Облагается взносами» = 1, если это зарплата штатного сотрудника. Пояснения к ячейкам минимального сценария — в комментариях.</t>
         </is>
       </c>
     </row>
@@ -1259,7 +1299,7 @@
         </is>
       </c>
       <c r="B14" s="19" t="n">
-        <v>15000</v>
+        <v>300</v>
       </c>
       <c r="C14" s="19" t="n">
         <v>30000</v>
@@ -1278,7 +1318,7 @@
         </is>
       </c>
       <c r="B15" s="19" t="n">
-        <v>15000</v>
+        <v>0</v>
       </c>
       <c r="C15" s="19" t="n">
         <v>40000</v>
@@ -1297,7 +1337,7 @@
         </is>
       </c>
       <c r="B16" s="19" t="n">
-        <v>8000</v>
+        <v>770</v>
       </c>
       <c r="C16" s="19" t="n">
         <v>15000</v>
@@ -1316,7 +1356,7 @@
         </is>
       </c>
       <c r="B17" s="19" t="n">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="C17" s="19" t="n">
         <v>90000</v>
@@ -1392,7 +1432,7 @@
         </is>
       </c>
       <c r="B21" s="19" t="n">
-        <v>7000</v>
+        <v>0</v>
       </c>
       <c r="C21" s="19" t="n">
         <v>10000</v>
@@ -1411,7 +1451,7 @@
         </is>
       </c>
       <c r="B22" s="19" t="n">
-        <v>40000</v>
+        <v>0</v>
       </c>
       <c r="C22" s="19" t="n">
         <v>100000</v>
@@ -1458,6 +1498,7 @@
     <mergeCell ref="A2:F2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <legacyDrawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="anysvml"/>
 </worksheet>
 </file>
 

</xml_diff>